<commit_message>
feat(secteurs): rôle de LaNum, cibles REEN, civic tech, accessibilité et IA
- Rôle de LaNum Pays Basque reformulé partout : elle propose ces versions
  alternatives pour les publics qu'elle accompagne dans le projet
  européen NÉONUM ; co-édition avec l'INR
- Collectivités : C.5 recentrée sur la stratégie numérique responsable de
  la loi REEN ; C.2 cite conseillers numériques, France Services et
  Aidants Connect ; nouvelles cibles C.6 accessibilité des contenus et de
  l'accueil, C.7 recensement et encadrement de l'IA, C.8 civic tech et
  participation citoyenne
- Feuille « Cibles métier » copiée de l'onglet ONR qui a juste assez de
  lignes (lignes en trop masquées), avec zone d'impression et titres
- Logos : un seul bandeau INR + LaNum + NÉONUM remplace le logo INR, plus
  de chevauchement dans OnlyOffice
- Hauteur des lignes de cibles ajustée à la longueur des libellés

Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
+++ b/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
@@ -63,6 +63,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="7">'ONR 5'!$B$2:$V$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'ONR 5'!$4:$6,'ONR 5'!$B:$C</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'Résultats synthèse'!$B$2:$M$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Cibles métier'!$B$2:$V$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Cibles métier'!$4:$6,'Cibles métier'!$B:$C</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1" calcMode="auto" forceFullCalc="1"/>
   <fileRecoveryPr autoRecover="0"/>
@@ -456,10 +458,11 @@
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>Utilisateur invité</author>
     <author>Utilisateur</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{EB80FB45-ED39-4EE0-B694-4C8CBE5F9519}">
       <text>
         <r>
           <rPr>
@@ -467,47 +470,47 @@
             <color rgb="FF000000"/>
             <rFont val="Helv"/>
           </rPr>
-          <t>Parce que les services numériques peuvent être sources d’exclusion sociale, d’individualisation et d’obsolescence matérielle et logicielle, nous nous engageons à développer des offres de services accessibles pour tous, inclusives et durables.</t>
+          <t>Parce que le numérique est un acteur majeur d’émissions de Gaz à Effet de Serre, d’épuisement des ressources et d’affaissement de la biodiversité, participant activement au changement climatique, nous nous engageons à optimiser les outils numériques pour limiter leurs impacts et consommations.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
+    <comment ref="D5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <t>Décrire les opportunités et les menaces associées à cette cible pour l’organisation : enjeux économiques, sociaux, environnementaux, réglementaires ou opérationnels.</t>
       </text>
     </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000003000000}">
+    <comment ref="E5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <t>Évaluer l’importance de la cible pour l’organisation.
 0 : non applicable ; 1 : peu importante ; 2 : importante ; 3 : très importante.
 Une importance de 0 classe la cible comme non applicable, même sans note de performance.</t>
       </text>
     </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
+    <comment ref="F5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <t>Évaluer la situation actuelle à partir d’éléments documentés.
 1 : pas du tout atteinte ; 2 : atteinte en partie ; 3 : en voie d’être atteinte ; 4 : atteinte.
 Laisser vide si la cible n’est pas évaluée ou n’est pas applicable.</t>
       </text>
     </comment>
-    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000005000000}">
+    <comment ref="G5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
       <text>
         <t>Justifier la note de performance avec les mesures déjà en place, les résultats observés, les indicateurs disponibles et les sources datées. Distinguer les actions réalisées des actions seulement prévues.</t>
       </text>
     </comment>
-    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000007000000}">
+    <comment ref="I5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <t>Décrire les forces et les faiblesses internes : compétences, moyens humains, financiers et techniques, et partenaires disponibles pour agir sur la cible.</t>
       </text>
     </comment>
-    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000008000000}">
+    <comment ref="J5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
       <text>
         <t>Calcul automatique à partir de l’importance et de la performance, selon la matrice de l’onglet Priorisation.
 Importance 0 : non applicable. Sinon, deux notes valides sont nécessaires.
 Consulter Résultats détaillés et Résultats synthèse pour les résultats consolidés.</t>
       </text>
     </comment>
-    <comment ref="V5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-00000A000000}">
+    <comment ref="V5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000A000000}">
       <text>
         <t>Proposer des actions contribuant à l’atteinte de la cible. Préciser, si possible, un responsable, une échéance et un résultat attendu.
 Une proposition renseignée ne signifie pas que l’action a été validée ou réalisée.</t>
@@ -27544,7 +27547,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Version « Collectivités territoriales » co-éditée par l'Institut du Numérique Responsable (INR) et LaNum Pays Basque, dans le cadre du projet NÉONUM, d'après la GPC-ONR de l'INR. Les cibles métier (feuille « Cibles métier ») ne sont pas reprises dans les feuilles de résultats.</a:t>
+            <a:t>Version « Collectivités territoriales » proposée par LaNum Pays Basque pour les publics qu'elle accompagne dans le projet européen NÉONUM, et co-éditée avec l'INR, d'après la GPC-ONR. Les cibles métier (feuille « Cibles métier ») ne sont pas reprises dans les feuilles de résultats.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -27569,76 +27572,22 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="57e11928-67da-43e8-bf4d-cd8442aff663"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="officialLogoINR20261007"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="bandeauCoedition"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -30094,76 +30043,22 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="9bd40fee-3145-48bd-b262-f6546a52b031"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="officialLogoINR20261007"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="bandeauCoedition"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -30378,75 +30273,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a59bba7-19d6-49ba-821e-248463433195"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd0f8b23f0a7a4abc"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30524,75 +30365,21 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498475</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="966d4c1d-e16d-4837-80a0-1444665fbe1b"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4133cfea2974438b"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>135109</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>875913</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30615,70 +30402,16 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ad6eca7f-2512-4327-a38b-5fd4332cec7e"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R88a94acdc061494d"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30696,75 +30429,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>7156450</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="253580d9-a043-4736-af34-c3bf36bb7bd2"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1641b25ecc3940ba"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>5907259</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>8419713</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30782,75 +30461,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="5ba0819c-73d0-49f8-9222-16d663e15aa0"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R34c26571c7014388"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1182859</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30868,75 +30493,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a59bba7-19d6-49ba-821e-248463433195"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd0f8b23f0a7a4abc"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30954,75 +30525,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1b76089d-f7b4-461a-bc2a-0b97e5c05474"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf6467eda94464bb5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31040,75 +30557,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="9b925086-4e52-4a38-8282-40c16f0a476c"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5e03a6a319674c4e"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31126,75 +30589,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="67e8ff89-b205-4e84-b992-af3db7ffe8a1"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R009525bc9d6e404c"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31212,75 +30621,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>39</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>212725</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e81248c7-2f0d-494e-9b17-442281be75de"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8c85558606f24767"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>468484</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>723513</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -42545,7 +41900,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
-    <x:tabColor theme="9"/>
+    <x:tabColor theme="4"/>
     <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="12"/>
@@ -42561,8 +41916,8 @@
     <x:col min="9" max="9" width="32" style="871" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="23" style="871" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="5.6640625" style="866" hidden="1" customWidth="1"/>
-    <x:col min="12" max="12" width="5.6640625" style="866" hidden="1" customWidth="1"/>
-    <x:col min="13" max="13" width="5.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="12" max="12" width="16.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="13" max="13" width="17.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="14" max="14" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="15" max="15" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="16" max="16" width="5.6640625" style="866" hidden="1" customWidth="1"/>
@@ -42572,8 +41927,8 @@
     <x:col min="20" max="20" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="21" max="21" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="22" max="22" width="46" style="871" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="42.6640625" style="871" hidden="1" customWidth="1"/>
-    <x:col min="24" max="24" width="42.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="23" max="23" width="68.6640625" style="871" hidden="1" customWidth="1"/>
+    <x:col min="24" max="24" width="78.5" style="866" hidden="1" customWidth="1"/>
     <x:col min="25" max="25" width="10.6640625" style="866" customWidth="0" hidden="0"/>
     <x:col min="26" max="26" width="10.6640625" style="866" customWidth="0" hidden="0"/>
     <x:col min="27" max="27" width="10.6640625" style="866" customWidth="0" hidden="0"/>
@@ -42669,10 +42024,10 @@
     </x:row>
     <x:row r="4" ht="27" customHeight="1">
       <x:c r="A4" s="861"/>
-      <x:c r="B4" s="1822" t="str">
+      <x:c r="B4" s="1731" t="str">
         <x:v>Cibles à évaluer</x:v>
       </x:c>
-      <x:c r="C4" s="1823"/>
+      <x:c r="C4" s="1732"/>
       <x:c r="D4" s="1735" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Importance de la cible</x:t>
@@ -42715,8 +42070,8 @@
     </x:row>
     <x:row r="5" s="868" customFormat="1" ht="56" customHeight="1">
       <x:c r="A5" s="867"/>
-      <x:c r="B5" s="1824"/>
-      <x:c r="C5" s="1825"/>
+      <x:c r="B5" s="1733"/>
+      <x:c r="C5" s="1734"/>
       <x:c r="D5" s="1737" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Avantages possibles et risques</x:t>
@@ -42807,54 +42162,50 @@
           <x:t xml:space="preserve">Code priorité et compétences</x:t>
         </x:is>
       </x:c>
-      <x:c r="V5" s="1826" t="inlineStr">
+      <x:c r="V5" s="1751" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Actions proposées pour atteindre la cible</x:t>
         </x:is>
       </x:c>
-      <x:c r="W5" s="1753" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adhérence</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="W5" s="1752"/>
       <x:c r="X5" s="1753"/>
     </x:row>
     <x:row r="6" s="875" customFormat="1" ht="34" customHeight="1">
       <x:c r="A6" s="874"/>
-      <x:c r="B6" s="1832" t="str">
+      <x:c r="B6" s="1764" t="str">
         <x:v>Renseigner les cellules jaunes pour les notes, puis les textes utiles. La priorité se calcule automatiquement. Faire défiler vers la droite pour proposer des actions.</x:v>
       </x:c>
-      <x:c r="C6" s="1833"/>
-      <x:c r="D6" s="1834"/>
-      <x:c r="E6" s="1834"/>
-      <x:c r="F6" s="1834"/>
-      <x:c r="G6" s="1834"/>
-      <x:c r="H6" s="1834"/>
-      <x:c r="I6" s="1834"/>
-      <x:c r="J6" s="1834"/>
-      <x:c r="K6" s="1834"/>
-      <x:c r="L6" s="1834"/>
-      <x:c r="M6" s="1834"/>
-      <x:c r="N6" s="1834"/>
-      <x:c r="O6" s="1834"/>
-      <x:c r="P6" s="1834"/>
-      <x:c r="Q6" s="1834"/>
-      <x:c r="R6" s="1834"/>
-      <x:c r="S6" s="1834"/>
-      <x:c r="T6" s="1834"/>
-      <x:c r="U6" s="1834"/>
-      <x:c r="V6" s="1835"/>
-      <x:c r="W6" s="1836"/>
-      <x:c r="X6" s="1129"/>
+      <x:c r="C6" s="1765"/>
+      <x:c r="D6" s="1766"/>
+      <x:c r="E6" s="1766"/>
+      <x:c r="F6" s="1766"/>
+      <x:c r="G6" s="1766"/>
+      <x:c r="H6" s="1766"/>
+      <x:c r="I6" s="1766"/>
+      <x:c r="J6" s="1766"/>
+      <x:c r="K6" s="1766"/>
+      <x:c r="L6" s="1766"/>
+      <x:c r="M6" s="1766"/>
+      <x:c r="N6" s="1766"/>
+      <x:c r="O6" s="1766"/>
+      <x:c r="P6" s="1766"/>
+      <x:c r="Q6" s="1766"/>
+      <x:c r="R6" s="1766"/>
+      <x:c r="S6" s="1766"/>
+      <x:c r="T6" s="1766"/>
+      <x:c r="U6" s="1766"/>
+      <x:c r="V6" s="1766"/>
+      <x:c r="W6" s="1765"/>
+      <x:c r="X6" s="1107"/>
     </x:row>
-    <x:row r="7" s="952" customFormat="1" ht="70" customHeight="1">
+    <x:row r="7" s="952" customFormat="1" ht="76" customHeight="1">
       <x:c r="A7" s="951"/>
-      <x:c r="B7" s="1804" t="inlineStr">
+      <x:c r="B7" s="1803" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">C.1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="1796" t="inlineStr">
+      <x:c r="C7" s="1795" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Évaluer l'utilité environnementale et sociale des objets connectés et des projets de « territoire intelligent » avant de les déployer : capteurs, éclairage, vidéoprotection, plateformes de données.</x:t>
         </x:is>
@@ -42864,55 +42215,55 @@
       <x:c r="F7" s="1802"/>
       <x:c r="G7" s="1798"/>
       <x:c r="H7" s="1802"/>
-      <x:c r="I7" s="1798"/>
+      <x:c r="I7" s="1799"/>
       <x:c r="J7" s="1806" t="str">
-        <x:f t="shared" ref="J7:J9" si="0">S7</x:f>
-      </x:c>
-      <x:c r="K7" s="1783" t="str">
+        <x:f>S7</x:f>
+      </x:c>
+      <x:c r="K7" s="1777" t="str">
         <x:f>IF(IF(ISNUMBER(E7),AND(E7&gt;=0,E7&lt;=3,MOD(E7,1)=0),FALSE),IF(E7=0,0,IF(IF(ISNUMBER(F7),AND(F7&gt;=1,F7&lt;=4,MOD(F7,1)=0),FALSE),E7*10+F7,"")),"")</x:f>
       </x:c>
-      <x:c r="L7" s="1783" t="b">
+      <x:c r="L7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),K7=31,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M7" s="1783" t="b">
+      <x:c r="M7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=21,K7=32),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N7" s="1783" t="b">
+      <x:c r="N7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=22,K7=33),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O7" s="1783" t="b">
+      <x:c r="O7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=11,K7=12),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P7" s="1783" t="b">
+      <x:c r="P7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=23,K7=34),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q7" s="1783" t="b">
+      <x:c r="Q7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=13,K7=14,K7=24),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="R7" s="1783" t="b">
+      <x:c r="R7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),K7=0,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S7" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T7),INDEX($L$5:$R$5,1,7-T7),"")</x:f>
-      </x:c>
-      <x:c r="T7" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K7),IF(L7,6,IF(M7,5,IF(N7,4,IF(O7,3,IF(P7,2,IF(Q7,1,0)))))),"")</x:f>
-      </x:c>
-      <x:c r="U7" s="1783" t="str">
+      <x:c r="S7" s="1777" t="str">
+        <x:f t="shared" ref="S7:S12" si="0">IF(ISNUMBER(T7),INDEX($L$5:$R$5,1,7-T7),"")</x:f>
+      </x:c>
+      <x:c r="T7" s="1777" t="str">
+        <x:f t="shared" ref="T7:T12" si="1">IF(ISNUMBER(K7),IF(L7,6,IF(M7,5,IF(N7,4,IF(O7,3,IF(P7,2,IF(Q7,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U7" s="1790" t="str">
         <x:f>IF(AND(ISNUMBER(T7),ISNUMBER(H7)),IF(AND(H7&gt;=1,H7&lt;=4,MOD(H7,1)=0),T7*10+H7,""),"")</x:f>
       </x:c>
-      <x:c r="V7" s="1798"/>
-      <x:c r="W7" s="1123"/>
-      <x:c r="X7" s="1113"/>
+      <x:c r="V7" s="1799"/>
+      <x:c r="W7" s="1103"/>
+      <x:c r="X7" s="903"/>
     </x:row>
-    <x:row r="8" s="952" customFormat="1" ht="76" customHeight="1">
+    <x:row r="8" s="952" customFormat="1" ht="77" customHeight="1">
       <x:c r="A8" s="951"/>
       <x:c r="B8" s="1804" t="inlineStr">
         <x:is>
@@ -42921,7 +42272,7 @@
       </x:c>
       <x:c r="C8" s="1796" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lutter contre l'illectronisme : financer la médiation numérique, garder un accueil physique et une solution non numérique pour chaque démarche.</x:t>
+          <x:t xml:space="preserve">Lutter contre l'illectronisme : soutenir la médiation numérique (conseillers numériques, espaces France Services, Aidants Connect), garder un accueil physique et une solution non numérique pour chaque démarche.</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" s="1798"/>
@@ -42929,53 +42280,53 @@
       <x:c r="F8" s="1802"/>
       <x:c r="G8" s="1798"/>
       <x:c r="H8" s="1802"/>
-      <x:c r="I8" s="1798"/>
+      <x:c r="I8" s="1799"/>
       <x:c r="J8" s="1806" t="str">
-        <x:f t="shared" si="0">S8</x:f>
-      </x:c>
-      <x:c r="K8" s="1783" t="str">
-        <x:f>IF(IF(ISNUMBER(E8),AND(E8&gt;=0,E8&lt;=3,MOD(E8,1)=0),FALSE),IF(E8=0,0,IF(IF(ISNUMBER(F8),AND(F8&gt;=1,F8&lt;=4,MOD(F8,1)=0),FALSE),E8*10+F8,"")),"")</x:f>
-      </x:c>
-      <x:c r="L8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),K8=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=21,K8=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=22,K8=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=11,K8=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=23,K8=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=13,K8=14,K8=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),K8=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S8" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T8),INDEX($L$5:$R$5,1,7-T8),"")</x:f>
-      </x:c>
-      <x:c r="T8" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K8),IF(L8,6,IF(M8,5,IF(N8,4,IF(O8,3,IF(P8,2,IF(Q8,1,0)))))),"")</x:f>
-      </x:c>
-      <x:c r="U8" s="1783" t="str">
-        <x:f>IF(AND(ISNUMBER(T8),ISNUMBER(H8)),IF(AND(H8&gt;=1,H8&lt;=4,MOD(H8,1)=0),T8*10+H8,""),"")</x:f>
-      </x:c>
-      <x:c r="V8" s="1798"/>
-      <x:c r="W8" s="1109"/>
-      <x:c r="X8" s="1108"/>
+        <x:f t="shared" ref="J8:J12" si="2">S8</x:f>
+      </x:c>
+      <x:c r="K8" s="1777" t="str">
+        <x:f t="shared" ref="K8:K12" si="3">IF(IF(ISNUMBER(E8),AND(E8&gt;=0,E8&lt;=3,MOD(E8,1)=0),FALSE),IF(E8=0,0,IF(IF(ISNUMBER(F8),AND(F8&gt;=1,F8&lt;=4,MOD(F8,1)=0),FALSE),E8*10+F8,"")),"")</x:f>
+      </x:c>
+      <x:c r="L8" s="1777" t="b">
+        <x:f t="shared" ref="L8:L12" si="4">IF(ISNUMBER(K8),K8=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="1777" t="b">
+        <x:f t="shared" ref="M8:M12" si="5">IF(ISNUMBER(K8),OR(K8=21,K8=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="1777" t="b">
+        <x:f t="shared" ref="N8:N12" si="6">IF(ISNUMBER(K8),OR(K8=22,K8=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="1777" t="b">
+        <x:f t="shared" ref="O8:O12" si="7">IF(ISNUMBER(K8),OR(K8=11,K8=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P8" s="1777" t="b">
+        <x:f t="shared" ref="P8:P12" si="8">IF(ISNUMBER(K8),OR(K8=23,K8=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="1777" t="b">
+        <x:f t="shared" ref="Q8:Q12" si="9">IF(ISNUMBER(K8),OR(K8=13,K8=14,K8=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R8" s="1777" t="b">
+        <x:f t="shared" ref="R8:R12" si="10">IF(ISNUMBER(K8),K8=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="1777" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T8),INDEX($L$5:$R$5,1,7-T8),"")</x:f>
+      </x:c>
+      <x:c r="T8" s="1777" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K8),IF(L8,6,IF(M8,5,IF(N8,4,IF(O8,3,IF(P8,2,IF(Q8,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U8" s="1790" t="str">
+        <x:f t="shared" ref="U8:U12" si="11">IF(AND(ISNUMBER(T8),ISNUMBER(H8)),IF(AND(H8&gt;=1,H8&lt;=4,MOD(H8,1)=0),T8*10+H8,""),"")</x:f>
+      </x:c>
+      <x:c r="V8" s="1799"/>
+      <x:c r="W8" s="1118"/>
+      <x:c r="X8" s="1117"/>
     </x:row>
     <x:row r="9" s="952" customFormat="1" ht="76" customHeight="1">
       <x:c r="A9" s="951"/>
@@ -42994,53 +42345,53 @@
       <x:c r="F9" s="1802"/>
       <x:c r="G9" s="1798"/>
       <x:c r="H9" s="1802"/>
-      <x:c r="I9" s="1798"/>
+      <x:c r="I9" s="1799"/>
       <x:c r="J9" s="1806" t="str">
-        <x:f t="shared" si="0">S9</x:f>
+        <x:f t="shared" si="2">S9</x:f>
       </x:c>
       <x:c r="K9" s="1783" t="str">
-        <x:f>IF(IF(ISNUMBER(E9),AND(E9&gt;=0,E9&lt;=3,MOD(E9,1)=0),FALSE),IF(E9=0,0,IF(IF(ISNUMBER(F9),AND(F9&gt;=1,F9&lt;=4,MOD(F9,1)=0),FALSE),E9*10+F9,"")),"")</x:f>
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E9),AND(E9&gt;=0,E9&lt;=3,MOD(E9,1)=0),FALSE),IF(E9=0,0,IF(IF(ISNUMBER(F9),AND(F9&gt;=1,F9&lt;=4,MOD(F9,1)=0),FALSE),E9*10+F9,"")),"")</x:f>
       </x:c>
       <x:c r="L9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),K9=31,FALSE)</x:f>
+        <x:f t="shared" si="4">IF(ISNUMBER(K9),K9=31,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=21,K9=32),FALSE)</x:f>
+        <x:f t="shared" si="5">IF(ISNUMBER(K9),OR(K9=21,K9=32),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=22,K9=33),FALSE)</x:f>
+        <x:f t="shared" si="6">IF(ISNUMBER(K9),OR(K9=22,K9=33),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=11,K9=12),FALSE)</x:f>
+        <x:f t="shared" si="7">IF(ISNUMBER(K9),OR(K9=11,K9=12),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=23,K9=34),FALSE)</x:f>
+        <x:f t="shared" si="8">IF(ISNUMBER(K9),OR(K9=23,K9=34),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=13,K9=14,K9=24),FALSE)</x:f>
+        <x:f t="shared" si="9">IF(ISNUMBER(K9),OR(K9=13,K9=14,K9=24),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),K9=0,FALSE)</x:f>
+        <x:f t="shared" si="10">IF(ISNUMBER(K9),K9=0,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S9" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T9),INDEX($L$5:$R$5,1,7-T9),"")</x:f>
+        <x:f t="shared" si="0">IF(ISNUMBER(T9),INDEX($L$5:$R$5,1,7-T9),"")</x:f>
       </x:c>
       <x:c r="T9" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K9),IF(L9,6,IF(M9,5,IF(N9,4,IF(O9,3,IF(P9,2,IF(Q9,1,0)))))),"")</x:f>
+        <x:f t="shared" si="1">IF(ISNUMBER(K9),IF(L9,6,IF(M9,5,IF(N9,4,IF(O9,3,IF(P9,2,IF(Q9,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U9" s="1783" t="str">
-        <x:f>IF(AND(ISNUMBER(T9),ISNUMBER(H9)),IF(AND(H9&gt;=1,H9&lt;=4,MOD(H9,1)=0),T9*10+H9,""),"")</x:f>
-      </x:c>
-      <x:c r="V9" s="1798"/>
-      <x:c r="W9" s="1122"/>
-      <x:c r="X9" s="1114"/>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T9),ISNUMBER(H9)),IF(AND(H9&gt;=1,H9&lt;=4,MOD(H9,1)=0),T9*10+H9,""),"")</x:f>
+      </x:c>
+      <x:c r="V9" s="1799"/>
+      <x:c r="W9" s="1104"/>
+      <x:c r="X9" s="1116"/>
     </x:row>
     <x:row r="10" s="952" customFormat="1" ht="70" customHeight="1">
       <x:c r="A10" s="951"/>
@@ -43059,64 +42410,64 @@
       <x:c r="F10" s="1802"/>
       <x:c r="G10" s="1798"/>
       <x:c r="H10" s="1802"/>
-      <x:c r="I10" s="1798"/>
+      <x:c r="I10" s="1799"/>
       <x:c r="J10" s="1806" t="str">
-        <x:f>S10</x:f>
-      </x:c>
-      <x:c r="K10" s="1777" t="str">
-        <x:f>IF(IF(ISNUMBER(E10),AND(E10&gt;=0,E10&lt;=3,MOD(E10,1)=0),FALSE),IF(E10=0,0,IF(IF(ISNUMBER(F10),AND(F10&gt;=1,F10&lt;=4,MOD(F10,1)=0),FALSE),E10*10+F10,"")),"")</x:f>
-      </x:c>
-      <x:c r="L10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),K10=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=21,K10=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=22,K10=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=11,K10=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=23,K10=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=13,K10=14,K10=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),K10=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S10" s="1777" t="str">
-        <x:f>IF(ISNUMBER(T10),INDEX($L$5:$R$5,1,7-T10),"")</x:f>
-      </x:c>
-      <x:c r="T10" s="1777" t="str">
-        <x:f>IF(ISNUMBER(K10),IF(L10,6,IF(M10,5,IF(N10,4,IF(O10,3,IF(P10,2,IF(Q10,1,0)))))),"")</x:f>
+        <x:f t="shared" si="2">S10</x:f>
+      </x:c>
+      <x:c r="K10" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E10),AND(E10&gt;=0,E10&lt;=3,MOD(E10,1)=0),FALSE),IF(E10=0,0,IF(IF(ISNUMBER(F10),AND(F10&gt;=1,F10&lt;=4,MOD(F10,1)=0),FALSE),E10*10+F10,"")),"")</x:f>
+      </x:c>
+      <x:c r="L10" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K10),K10=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K10),OR(K10=21,K10=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K10),OR(K10=22,K10=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K10),OR(K10=11,K10=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P10" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K10),OR(K10=23,K10=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K10),OR(K10=13,K10=14,K10=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R10" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K10),K10=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T10),INDEX($L$5:$R$5,1,7-T10),"")</x:f>
+      </x:c>
+      <x:c r="T10" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K10),IF(L10,6,IF(M10,5,IF(N10,4,IF(O10,3,IF(P10,2,IF(Q10,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U10" s="1790" t="str">
-        <x:f>IF(AND(ISNUMBER(T10),ISNUMBER(H10)),IF(AND(H10&gt;=1,H10&lt;=4,MOD(H10,1)=0),T10*10+H10,""),"")</x:f>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T10),ISNUMBER(H10)),IF(AND(H10&gt;=1,H10&lt;=4,MOD(H10,1)=0),T10*10+H10,""),"")</x:f>
       </x:c>
       <x:c r="V10" s="1798"/>
-      <x:c r="W10" s="1109"/>
-      <x:c r="X10" s="1108"/>
+      <x:c r="W10" s="1105"/>
+      <x:c r="X10" s="903"/>
     </x:row>
-    <x:row r="11" s="952" customFormat="1" ht="70" customHeight="1">
+    <x:row r="11" s="952" customFormat="1" ht="100" customHeight="1">
       <x:c r="A11" s="951"/>
-      <x:c r="B11" s="1804" t="inlineStr">
+      <x:c r="B11" s="1805" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">C.5</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="1796" t="inlineStr">
+      <x:c r="C11" s="1797" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Former les élus et les agents au numérique responsable, et l'inscrire dans la stratégie numérique responsable prévue par la loi REEN.</x:t>
+          <x:t xml:space="preserve">Adopter et faire vivre la stratégie numérique responsable prévue par la loi REEN : obligatoire pour les communes et intercommunalités de plus de 50 000 habitants, recommandée pour les autres. Fixer des objectifs de réduction de l'empreinte du numérique, suivre leur mise en œuvre et former les élus et les agents.</x:t>
         </x:is>
       </x:c>
       <x:c r="D11" s="1798"/>
@@ -43124,98 +42475,289 @@
       <x:c r="F11" s="1802"/>
       <x:c r="G11" s="1798"/>
       <x:c r="H11" s="1802"/>
-      <x:c r="I11" s="1798"/>
-      <x:c r="J11" s="1806" t="n">
-        <x:f>S11</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K11" s="1777" t="str">
-        <x:f>IF(IF(ISNUMBER(E11),AND(E11&gt;=0,E11&lt;=3,MOD(E11,1)=0),FALSE),IF(E11=0,0,IF(IF(ISNUMBER(F11),AND(F11&gt;=1,F11&lt;=4,MOD(F11,1)=0),FALSE),E11*10+F11,"")),"")</x:f>
-      </x:c>
-      <x:c r="L11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),K11=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=21,K11=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=22,K11=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=11,K11=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=23,K11=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=13,K11=14,K11=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),K11=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S11" s="1777" t="str">
-        <x:f>IF(ISNUMBER(T11),INDEX($L$5:$R$5,1,7-T11),"")</x:f>
-      </x:c>
-      <x:c r="T11" s="1777" t="str">
-        <x:f>IF(ISNUMBER(K11),IF(L11,6,IF(M11,5,IF(N11,4,IF(O11,3,IF(P11,2,IF(Q11,1,0)))))),"")</x:f>
+      <x:c r="I11" s="1799"/>
+      <x:c r="J11" s="1806" t="str">
+        <x:f t="shared" si="2">S11</x:f>
+      </x:c>
+      <x:c r="K11" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E11),AND(E11&gt;=0,E11&lt;=3,MOD(E11,1)=0),FALSE),IF(E11=0,0,IF(IF(ISNUMBER(F11),AND(F11&gt;=1,F11&lt;=4,MOD(F11,1)=0),FALSE),E11*10+F11,"")),"")</x:f>
+      </x:c>
+      <x:c r="L11" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K11),K11=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K11),OR(K11=21,K11=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K11),OR(K11=22,K11=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K11),OR(K11=11,K11=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P11" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K11),OR(K11=23,K11=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q11" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K11),OR(K11=13,K11=14,K11=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R11" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K11),K11=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T11),INDEX($L$5:$R$5,1,7-T11),"")</x:f>
+      </x:c>
+      <x:c r="T11" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K11),IF(L11,6,IF(M11,5,IF(N11,4,IF(O11,3,IF(P11,2,IF(Q11,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U11" s="1790" t="str">
-        <x:f>IF(AND(ISNUMBER(T11),ISNUMBER(H11)),IF(AND(H11&gt;=1,H11&lt;=4,MOD(H11,1)=0),T11*10+H11,""),"")</x:f>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T11),ISNUMBER(H11)),IF(AND(H11&gt;=1,H11&lt;=4,MOD(H11,1)=0),T11*10+H11,""),"")</x:f>
       </x:c>
       <x:c r="V11" s="1798"/>
-      <x:c r="W11" s="1109"/>
-      <x:c r="X11" s="1108"/>
+      <x:c r="W11" s="1119"/>
+      <x:c r="X11" s="1114"/>
     </x:row>
-    <x:row r="12">
-      <x:c r="V12" s="893"/>
+    <x:row r="12" s="953" customFormat="1" ht="100" customHeight="1">
+      <x:c r="A12" s="951"/>
+      <x:c r="B12" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rendre accessibles les contenus que la collectivité produit chaque jour : documents, publications sur les réseaux sociaux, vidéos sous-titrées, textes en facile à lire et à comprendre (FALC). Former les agents qui les produisent et offrir un accueil accessible, y compris aux personnes sourdes et malentendantes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="1798"/>
+      <x:c r="E12" s="1802"/>
+      <x:c r="F12" s="1802"/>
+      <x:c r="G12" s="1798"/>
+      <x:c r="H12" s="1802"/>
+      <x:c r="I12" s="1799"/>
+      <x:c r="J12" s="1806" t="str">
+        <x:f t="shared" si="2">S12</x:f>
+      </x:c>
+      <x:c r="K12" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E12),AND(E12&gt;=0,E12&lt;=3,MOD(E12,1)=0),FALSE),IF(E12=0,0,IF(IF(ISNUMBER(F12),AND(F12&gt;=1,F12&lt;=4,MOD(F12,1)=0),FALSE),E12*10+F12,"")),"")</x:f>
+      </x:c>
+      <x:c r="L12" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K12),K12=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K12),OR(K12=21,K12=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K12),OR(K12=22,K12=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K12),OR(K12=11,K12=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P12" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K12),OR(K12=23,K12=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q12" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K12),OR(K12=13,K12=14,K12=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R12" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K12),K12=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T12),INDEX($L$5:$R$5,1,7-T12),"")</x:f>
+      </x:c>
+      <x:c r="T12" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K12),IF(L12,6,IF(M12,5,IF(N12,4,IF(O12,3,IF(P12,2,IF(Q12,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U12" s="1790" t="str">
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T12),ISNUMBER(H12)),IF(AND(H12&gt;=1,H12&lt;=4,MOD(H12,1)=0),T12*10+H12,""),"")</x:f>
+      </x:c>
+      <x:c r="V12" s="1798"/>
+      <x:c r="W12" s="1120"/>
+      <x:c r="X12" s="1114"/>
+    </x:row>
+    <x:row r="13" ht="88.5" customHeight="1">
+      <x:c r="B13" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Recenser les usages de l'intelligence artificielle dans la collectivité, y compris l'IA générative utilisée par les agents. Les encadrer par une charte, vérifier les obligations du règlement européen sur l'IA, et informer les habitants des usages qui les concernent.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="1798"/>
+      <x:c r="E13" s="1802"/>
+      <x:c r="F13" s="1802"/>
+      <x:c r="G13" s="1798"/>
+      <x:c r="H13" s="1802"/>
+      <x:c r="I13" s="1799"/>
+      <x:c r="J13" s="1806" t="str">
+        <x:f t="shared" ref="J13" si="12">S13</x:f>
+      </x:c>
+      <x:c r="K13" s="1786" t="str">
+        <x:f t="shared" ref="K13" si="13">IF(IF(ISNUMBER(E13),AND(E13&gt;=0,E13&lt;=3,MOD(E13,1)=0),FALSE),IF(E13=0,0,IF(IF(ISNUMBER(F13),AND(F13&gt;=1,F13&lt;=4,MOD(F13,1)=0),FALSE),E13*10+F13,"")),"")</x:f>
+      </x:c>
+      <x:c r="L13" s="1786" t="b">
+        <x:f t="shared" ref="L13" si="14">IF(ISNUMBER(K13),K13=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="1786" t="b">
+        <x:f t="shared" ref="M13" si="15">IF(ISNUMBER(K13),OR(K13=21,K13=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="1786" t="b">
+        <x:f t="shared" ref="N13" si="16">IF(ISNUMBER(K13),OR(K13=22,K13=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="1786" t="b">
+        <x:f t="shared" ref="O13" si="17">IF(ISNUMBER(K13),OR(K13=11,K13=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P13" s="1786" t="b">
+        <x:f t="shared" ref="P13" si="18">IF(ISNUMBER(K13),OR(K13=23,K13=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q13" s="1786" t="b">
+        <x:f t="shared" ref="Q13" si="19">IF(ISNUMBER(K13),OR(K13=13,K13=14,K13=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R13" s="1786" t="b">
+        <x:f t="shared" ref="R13" si="20">IF(ISNUMBER(K13),K13=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="1786" t="str">
+        <x:f t="shared" ref="S13" si="21">IF(ISNUMBER(T13),INDEX($L$5:$R$5,1,7-T13),"")</x:f>
+      </x:c>
+      <x:c r="T13" s="1786" t="str">
+        <x:f t="shared" ref="T13" si="22">IF(ISNUMBER(K13),IF(L13,6,IF(M13,5,IF(N13,4,IF(O13,3,IF(P13,2,IF(Q13,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U13" s="1790" t="str">
+        <x:f t="shared" ref="U13" si="23">IF(AND(ISNUMBER(T13),ISNUMBER(H13)),IF(AND(H13&gt;=1,H13&lt;=4,MOD(H13,1)=0),T13*10+H13,""),"")</x:f>
+      </x:c>
+      <x:c r="V13" s="1798"/>
+      <x:c r="W13" s="1121"/>
+      <x:c r="X13" s="1114"/>
+    </x:row>
+    <x:row r="14" ht="88.5" customHeight="1">
+      <x:c r="B14" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Ouvrir la décision publique avec des outils de participation citoyenne (civic tech) : consultations, budgets participatifs, signalements. Choisir des outils ouverts, accessibles et sobres, comme les logiciels libres, et les compléter par des temps d'échange en présentiel.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="1798"/>
+      <x:c r="E14" s="1802"/>
+      <x:c r="F14" s="1802"/>
+      <x:c r="G14" s="1798"/>
+      <x:c r="H14" s="1802"/>
+      <x:c r="I14" s="1799"/>
+      <x:c r="J14" s="1806" t="n">
+        <x:f>S14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" s="1786" t="str">
+        <x:f>IF(IF(ISNUMBER(E14),AND(E14&gt;=0,E14&lt;=3,MOD(E14,1)=0),FALSE),IF(E14=0,0,IF(IF(ISNUMBER(F14),AND(F14&gt;=1,F14&lt;=4,MOD(F14,1)=0),FALSE),E14*10+F14,"")),"")</x:f>
+      </x:c>
+      <x:c r="L14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),K14=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=21,K14=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=22,K14=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=11,K14=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=23,K14=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=13,K14=14,K14=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),K14=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S14" s="1786" t="str">
+        <x:f>IF(ISNUMBER(T14),INDEX($L$5:$R$5,1,7-T14),"")</x:f>
+      </x:c>
+      <x:c r="T14" s="1786" t="str">
+        <x:f>IF(ISNUMBER(K14),IF(L14,6,IF(M14,5,IF(N14,4,IF(O14,3,IF(P14,2,IF(Q14,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U14" s="1790" t="str">
+        <x:f>IF(AND(ISNUMBER(T14),ISNUMBER(H14)),IF(AND(H14&gt;=1,H14&lt;=4,MOD(H14,1)=0),T14*10+H14,""),"")</x:f>
+      </x:c>
+      <x:c r="V14" s="1798"/>
+      <x:c r="W14" s="1121"/>
+      <x:c r="X14" s="1114"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="V4:X4"/>
+    <x:mergeCell ref="B6:W6"/>
     <x:mergeCell ref="B4:C5"/>
     <x:mergeCell ref="D4:E4"/>
     <x:mergeCell ref="F4:G4"/>
     <x:mergeCell ref="H4:I4"/>
+    <x:mergeCell ref="V4:X4"/>
     <x:mergeCell ref="B2:J3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="J7:J11">
-    <x:cfRule type="expression" dxfId="1633" priority="498">
+  <x:conditionalFormatting sqref="J7:J14">
+    <x:cfRule type="expression" dxfId="1626" priority="271">
       <x:formula>AND(ISNUMBER($T7),$T7=6)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1634" priority="499">
+    <x:cfRule type="expression" dxfId="1627" priority="272">
       <x:formula>AND(ISNUMBER($T7),$T7=5)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1635" priority="500">
+    <x:cfRule type="expression" dxfId="1628" priority="273">
       <x:formula>AND(ISNUMBER($T7),$T7=4)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1636" priority="501">
+    <x:cfRule type="expression" dxfId="1629" priority="274">
       <x:formula>AND(ISNUMBER($T7),$T7=3)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1637" priority="502">
+    <x:cfRule type="expression" dxfId="1630" priority="275">
       <x:formula>AND(ISNUMBER($T7),$T7=2)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1638" priority="503">
+    <x:cfRule type="expression" dxfId="1631" priority="276">
       <x:formula>AND(ISNUMBER($T7),$T7=1)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1639" priority="504">
+    <x:cfRule type="expression" dxfId="1632" priority="277">
       <x:formula>AND(ISNUMBER($T7),$T7=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="E7:E11" promptTitle="Importance de la cible" prompt="0 : non applicable&#10;1 : peu importante&#10;2 : importante&#10;3 : très importante&#10;Si 0, la performance peut rester vide." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="E7:E14" promptTitle="Importance de la cible" prompt="0 : non applicable&#10;1 : peu importante&#10;2 : importante&#10;3 : très importante&#10;Si 0, la performance peut rester vide." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"0,1,2,3"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="F7:F11" promptTitle="Performance actuelle" prompt="1 : pas du tout atteinte&#10;2 : atteinte en partie&#10;3 : en voie d’être atteinte&#10;4 : atteinte&#10;Laisser vide si non évaluée ou non applicable." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="F7:F14" promptTitle="Performance actuelle" prompt="1 : pas du tout atteinte&#10;2 : atteinte en partie&#10;3 : en voie d’être atteinte&#10;4 : atteinte&#10;Laisser vide si non évaluée ou non applicable." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"1,2,3,4"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="H7:H11" promptTitle="Compétences mobilisées" prompt="1 : équipe NR / RSE&#10;2 : NR / RSE et DSI&#10;3 : NR / RSE et équipe hors DSI&#10;4 : intervention extérieure" errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="H7:H14" promptTitle="Compétences mobilisées" prompt="1 : équipe NR / RSE&#10;2 : NR / RSE et DSI&#10;3 : NR / RSE et équipe hors DSI&#10;4 : intervention extérieure" errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"1,2,3,4"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
Rôle de LaNum (NÉONUM), cibles REEN, civic tech, accessibilité et IA, bandeau de logos (#15)
Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
+++ b/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
@@ -63,6 +63,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="7">'ONR 5'!$B$2:$V$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'ONR 5'!$4:$6,'ONR 5'!$B:$C</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'Résultats synthèse'!$B$2:$M$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Cibles métier'!$B$2:$V$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Cibles métier'!$4:$6,'Cibles métier'!$B:$C</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1" calcMode="auto" forceFullCalc="1"/>
   <fileRecoveryPr autoRecover="0"/>
@@ -456,10 +458,11 @@
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>Utilisateur invité</author>
     <author>Utilisateur</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{EB80FB45-ED39-4EE0-B694-4C8CBE5F9519}">
       <text>
         <r>
           <rPr>
@@ -467,47 +470,47 @@
             <color rgb="FF000000"/>
             <rFont val="Helv"/>
           </rPr>
-          <t>Parce que les services numériques peuvent être sources d’exclusion sociale, d’individualisation et d’obsolescence matérielle et logicielle, nous nous engageons à développer des offres de services accessibles pour tous, inclusives et durables.</t>
+          <t>Parce que le numérique est un acteur majeur d’émissions de Gaz à Effet de Serre, d’épuisement des ressources et d’affaissement de la biodiversité, participant activement au changement climatique, nous nous engageons à optimiser les outils numériques pour limiter leurs impacts et consommations.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
+    <comment ref="D5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <t>Décrire les opportunités et les menaces associées à cette cible pour l’organisation : enjeux économiques, sociaux, environnementaux, réglementaires ou opérationnels.</t>
       </text>
     </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000003000000}">
+    <comment ref="E5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <t>Évaluer l’importance de la cible pour l’organisation.
 0 : non applicable ; 1 : peu importante ; 2 : importante ; 3 : très importante.
 Une importance de 0 classe la cible comme non applicable, même sans note de performance.</t>
       </text>
     </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
+    <comment ref="F5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <t>Évaluer la situation actuelle à partir d’éléments documentés.
 1 : pas du tout atteinte ; 2 : atteinte en partie ; 3 : en voie d’être atteinte ; 4 : atteinte.
 Laisser vide si la cible n’est pas évaluée ou n’est pas applicable.</t>
       </text>
     </comment>
-    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000005000000}">
+    <comment ref="G5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
       <text>
         <t>Justifier la note de performance avec les mesures déjà en place, les résultats observés, les indicateurs disponibles et les sources datées. Distinguer les actions réalisées des actions seulement prévues.</t>
       </text>
     </comment>
-    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000007000000}">
+    <comment ref="I5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <t>Décrire les forces et les faiblesses internes : compétences, moyens humains, financiers et techniques, et partenaires disponibles pour agir sur la cible.</t>
       </text>
     </comment>
-    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000008000000}">
+    <comment ref="J5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
       <text>
         <t>Calcul automatique à partir de l’importance et de la performance, selon la matrice de l’onglet Priorisation.
 Importance 0 : non applicable. Sinon, deux notes valides sont nécessaires.
 Consulter Résultats détaillés et Résultats synthèse pour les résultats consolidés.</t>
       </text>
     </comment>
-    <comment ref="V5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-00000A000000}">
+    <comment ref="V5" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000A000000}">
       <text>
         <t>Proposer des actions contribuant à l’atteinte de la cible. Préciser, si possible, un responsable, une échéance et un résultat attendu.
 Une proposition renseignée ne signifie pas que l’action a été validée ou réalisée.</t>
@@ -27544,7 +27547,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Version « Collectivités territoriales » co-éditée par l'Institut du Numérique Responsable (INR) et LaNum Pays Basque, dans le cadre du projet NÉONUM, d'après la GPC-ONR de l'INR. Les cibles métier (feuille « Cibles métier ») ne sont pas reprises dans les feuilles de résultats.</a:t>
+            <a:t>Version « Collectivités territoriales » : LaNum Pays Basque l'a conçue pour les publics qu'elle accompagne dans le projet européen NÉONUM, à partir de la GPC-ONR ; l'INR la co-édite. Les feuilles de résultats ne reprennent pas les cibles de la feuille « Cibles métier ».</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -27569,76 +27572,22 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="57e11928-67da-43e8-bf4d-cd8442aff663"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="officialLogoINR20261007"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="bandeauCoedition"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -30094,76 +30043,22 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="9bd40fee-3145-48bd-b262-f6546a52b031"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="officialLogoINR20261007"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="bandeauCoedition"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -30378,75 +30273,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a59bba7-19d6-49ba-821e-248463433195"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd0f8b23f0a7a4abc"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30524,75 +30365,21 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498475</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="966d4c1d-e16d-4837-80a0-1444665fbe1b"/>
+        <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4133cfea2974438b"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>135109</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>875913</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30615,70 +30402,16 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ad6eca7f-2512-4327-a38b-5fd4332cec7e"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R88a94acdc061494d"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>708025</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>791604</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30696,75 +30429,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>7156450</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="253580d9-a043-4736-af34-c3bf36bb7bd2"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1641b25ecc3940ba"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>5907259</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>8419713</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30782,75 +30461,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="5ba0819c-73d0-49f8-9222-16d663e15aa0"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R34c26571c7014388"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1182859</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30868,75 +30493,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a59bba7-19d6-49ba-821e-248463433195"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd0f8b23f0a7a4abc"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -30954,75 +30525,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1b76089d-f7b4-461a-bc2a-0b97e5c05474"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf6467eda94464bb5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31040,75 +30557,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="9b925086-4e52-4a38-8282-40c16f0a476c"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5e03a6a319674c4e"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31126,75 +30589,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="67e8ff89-b205-4e84-b992-af3db7ffe8a1"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R009525bc9d6e404c"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>382759</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>380613</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -31212,75 +30621,21 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>39</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>212725</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2000250" cy="638175"/>
+    <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e81248c7-2f0d-494e-9b17-442281be75de"/>
+        <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8c85558606f24767"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>468484</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2299729" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="900" name="LaNum Pays Basque" descr="Logo LaNum Pays Basque"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>723513</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="778262" cy="638175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="901" name="NÉONUM" descr="Logo NÉONUM"/>
-        <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="logoCoediteur2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="bandeauCoedition"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -42545,7 +41900,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
-    <x:tabColor theme="9"/>
+    <x:tabColor theme="4"/>
     <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="12"/>
@@ -42561,8 +41916,8 @@
     <x:col min="9" max="9" width="32" style="871" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="23" style="871" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="5.6640625" style="866" hidden="1" customWidth="1"/>
-    <x:col min="12" max="12" width="5.6640625" style="866" hidden="1" customWidth="1"/>
-    <x:col min="13" max="13" width="5.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="12" max="12" width="16.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="13" max="13" width="17.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="14" max="14" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="15" max="15" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="16" max="16" width="5.6640625" style="866" hidden="1" customWidth="1"/>
@@ -42572,8 +41927,8 @@
     <x:col min="20" max="20" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="21" max="21" width="5.6640625" style="866" hidden="1" customWidth="1"/>
     <x:col min="22" max="22" width="46" style="871" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="42.6640625" style="871" hidden="1" customWidth="1"/>
-    <x:col min="24" max="24" width="42.6640625" style="866" hidden="1" customWidth="1"/>
+    <x:col min="23" max="23" width="68.6640625" style="871" hidden="1" customWidth="1"/>
+    <x:col min="24" max="24" width="78.5" style="866" hidden="1" customWidth="1"/>
     <x:col min="25" max="25" width="10.6640625" style="866" customWidth="0" hidden="0"/>
     <x:col min="26" max="26" width="10.6640625" style="866" customWidth="0" hidden="0"/>
     <x:col min="27" max="27" width="10.6640625" style="866" customWidth="0" hidden="0"/>
@@ -42669,10 +42024,10 @@
     </x:row>
     <x:row r="4" ht="27" customHeight="1">
       <x:c r="A4" s="861"/>
-      <x:c r="B4" s="1822" t="str">
+      <x:c r="B4" s="1731" t="str">
         <x:v>Cibles à évaluer</x:v>
       </x:c>
-      <x:c r="C4" s="1823"/>
+      <x:c r="C4" s="1732"/>
       <x:c r="D4" s="1735" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Importance de la cible</x:t>
@@ -42715,8 +42070,8 @@
     </x:row>
     <x:row r="5" s="868" customFormat="1" ht="56" customHeight="1">
       <x:c r="A5" s="867"/>
-      <x:c r="B5" s="1824"/>
-      <x:c r="C5" s="1825"/>
+      <x:c r="B5" s="1733"/>
+      <x:c r="C5" s="1734"/>
       <x:c r="D5" s="1737" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Avantages possibles et risques</x:t>
@@ -42807,54 +42162,50 @@
           <x:t xml:space="preserve">Code priorité et compétences</x:t>
         </x:is>
       </x:c>
-      <x:c r="V5" s="1826" t="inlineStr">
+      <x:c r="V5" s="1751" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Actions proposées pour atteindre la cible</x:t>
         </x:is>
       </x:c>
-      <x:c r="W5" s="1753" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adhérence</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="W5" s="1752"/>
       <x:c r="X5" s="1753"/>
     </x:row>
     <x:row r="6" s="875" customFormat="1" ht="34" customHeight="1">
       <x:c r="A6" s="874"/>
-      <x:c r="B6" s="1832" t="str">
+      <x:c r="B6" s="1764" t="str">
         <x:v>Renseigner les cellules jaunes pour les notes, puis les textes utiles. La priorité se calcule automatiquement. Faire défiler vers la droite pour proposer des actions.</x:v>
       </x:c>
-      <x:c r="C6" s="1833"/>
-      <x:c r="D6" s="1834"/>
-      <x:c r="E6" s="1834"/>
-      <x:c r="F6" s="1834"/>
-      <x:c r="G6" s="1834"/>
-      <x:c r="H6" s="1834"/>
-      <x:c r="I6" s="1834"/>
-      <x:c r="J6" s="1834"/>
-      <x:c r="K6" s="1834"/>
-      <x:c r="L6" s="1834"/>
-      <x:c r="M6" s="1834"/>
-      <x:c r="N6" s="1834"/>
-      <x:c r="O6" s="1834"/>
-      <x:c r="P6" s="1834"/>
-      <x:c r="Q6" s="1834"/>
-      <x:c r="R6" s="1834"/>
-      <x:c r="S6" s="1834"/>
-      <x:c r="T6" s="1834"/>
-      <x:c r="U6" s="1834"/>
-      <x:c r="V6" s="1835"/>
-      <x:c r="W6" s="1836"/>
-      <x:c r="X6" s="1129"/>
+      <x:c r="C6" s="1765"/>
+      <x:c r="D6" s="1766"/>
+      <x:c r="E6" s="1766"/>
+      <x:c r="F6" s="1766"/>
+      <x:c r="G6" s="1766"/>
+      <x:c r="H6" s="1766"/>
+      <x:c r="I6" s="1766"/>
+      <x:c r="J6" s="1766"/>
+      <x:c r="K6" s="1766"/>
+      <x:c r="L6" s="1766"/>
+      <x:c r="M6" s="1766"/>
+      <x:c r="N6" s="1766"/>
+      <x:c r="O6" s="1766"/>
+      <x:c r="P6" s="1766"/>
+      <x:c r="Q6" s="1766"/>
+      <x:c r="R6" s="1766"/>
+      <x:c r="S6" s="1766"/>
+      <x:c r="T6" s="1766"/>
+      <x:c r="U6" s="1766"/>
+      <x:c r="V6" s="1766"/>
+      <x:c r="W6" s="1765"/>
+      <x:c r="X6" s="1107"/>
     </x:row>
-    <x:row r="7" s="952" customFormat="1" ht="70" customHeight="1">
+    <x:row r="7" s="952" customFormat="1" ht="76" customHeight="1">
       <x:c r="A7" s="951"/>
-      <x:c r="B7" s="1804" t="inlineStr">
+      <x:c r="B7" s="1803" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">C.1</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="1796" t="inlineStr">
+      <x:c r="C7" s="1795" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Évaluer l'utilité environnementale et sociale des objets connectés et des projets de « territoire intelligent » avant de les déployer : capteurs, éclairage, vidéoprotection, plateformes de données.</x:t>
         </x:is>
@@ -42864,55 +42215,55 @@
       <x:c r="F7" s="1802"/>
       <x:c r="G7" s="1798"/>
       <x:c r="H7" s="1802"/>
-      <x:c r="I7" s="1798"/>
+      <x:c r="I7" s="1799"/>
       <x:c r="J7" s="1806" t="str">
-        <x:f t="shared" ref="J7:J9" si="0">S7</x:f>
-      </x:c>
-      <x:c r="K7" s="1783" t="str">
+        <x:f>S7</x:f>
+      </x:c>
+      <x:c r="K7" s="1777" t="str">
         <x:f>IF(IF(ISNUMBER(E7),AND(E7&gt;=0,E7&lt;=3,MOD(E7,1)=0),FALSE),IF(E7=0,0,IF(IF(ISNUMBER(F7),AND(F7&gt;=1,F7&lt;=4,MOD(F7,1)=0),FALSE),E7*10+F7,"")),"")</x:f>
       </x:c>
-      <x:c r="L7" s="1783" t="b">
+      <x:c r="L7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),K7=31,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M7" s="1783" t="b">
+      <x:c r="M7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=21,K7=32),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N7" s="1783" t="b">
+      <x:c r="N7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=22,K7=33),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O7" s="1783" t="b">
+      <x:c r="O7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=11,K7=12),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P7" s="1783" t="b">
+      <x:c r="P7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=23,K7=34),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q7" s="1783" t="b">
+      <x:c r="Q7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),OR(K7=13,K7=14,K7=24),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="R7" s="1783" t="b">
+      <x:c r="R7" s="1777" t="b">
         <x:f>IF(ISNUMBER(K7),K7=0,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S7" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T7),INDEX($L$5:$R$5,1,7-T7),"")</x:f>
-      </x:c>
-      <x:c r="T7" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K7),IF(L7,6,IF(M7,5,IF(N7,4,IF(O7,3,IF(P7,2,IF(Q7,1,0)))))),"")</x:f>
-      </x:c>
-      <x:c r="U7" s="1783" t="str">
+      <x:c r="S7" s="1777" t="str">
+        <x:f t="shared" ref="S7:S12" si="0">IF(ISNUMBER(T7),INDEX($L$5:$R$5,1,7-T7),"")</x:f>
+      </x:c>
+      <x:c r="T7" s="1777" t="str">
+        <x:f t="shared" ref="T7:T12" si="1">IF(ISNUMBER(K7),IF(L7,6,IF(M7,5,IF(N7,4,IF(O7,3,IF(P7,2,IF(Q7,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U7" s="1790" t="str">
         <x:f>IF(AND(ISNUMBER(T7),ISNUMBER(H7)),IF(AND(H7&gt;=1,H7&lt;=4,MOD(H7,1)=0),T7*10+H7,""),"")</x:f>
       </x:c>
-      <x:c r="V7" s="1798"/>
-      <x:c r="W7" s="1123"/>
-      <x:c r="X7" s="1113"/>
+      <x:c r="V7" s="1799"/>
+      <x:c r="W7" s="1103"/>
+      <x:c r="X7" s="903"/>
     </x:row>
-    <x:row r="8" s="952" customFormat="1" ht="76" customHeight="1">
+    <x:row r="8" s="952" customFormat="1" ht="77" customHeight="1">
       <x:c r="A8" s="951"/>
       <x:c r="B8" s="1804" t="inlineStr">
         <x:is>
@@ -42921,7 +42272,7 @@
       </x:c>
       <x:c r="C8" s="1796" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lutter contre l'illectronisme : financer la médiation numérique, garder un accueil physique et une solution non numérique pour chaque démarche.</x:t>
+          <x:t xml:space="preserve">Lutter contre l'illectronisme : soutenir la médiation numérique (conseillers numériques, espaces France Services, Aidants Connect), garder un accueil physique et une solution non numérique pour chaque démarche.</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" s="1798"/>
@@ -42929,53 +42280,53 @@
       <x:c r="F8" s="1802"/>
       <x:c r="G8" s="1798"/>
       <x:c r="H8" s="1802"/>
-      <x:c r="I8" s="1798"/>
+      <x:c r="I8" s="1799"/>
       <x:c r="J8" s="1806" t="str">
-        <x:f t="shared" si="0">S8</x:f>
-      </x:c>
-      <x:c r="K8" s="1783" t="str">
-        <x:f>IF(IF(ISNUMBER(E8),AND(E8&gt;=0,E8&lt;=3,MOD(E8,1)=0),FALSE),IF(E8=0,0,IF(IF(ISNUMBER(F8),AND(F8&gt;=1,F8&lt;=4,MOD(F8,1)=0),FALSE),E8*10+F8,"")),"")</x:f>
-      </x:c>
-      <x:c r="L8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),K8=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=21,K8=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=22,K8=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=11,K8=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=23,K8=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),OR(K8=13,K8=14,K8=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R8" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K8),K8=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S8" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T8),INDEX($L$5:$R$5,1,7-T8),"")</x:f>
-      </x:c>
-      <x:c r="T8" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K8),IF(L8,6,IF(M8,5,IF(N8,4,IF(O8,3,IF(P8,2,IF(Q8,1,0)))))),"")</x:f>
-      </x:c>
-      <x:c r="U8" s="1783" t="str">
-        <x:f>IF(AND(ISNUMBER(T8),ISNUMBER(H8)),IF(AND(H8&gt;=1,H8&lt;=4,MOD(H8,1)=0),T8*10+H8,""),"")</x:f>
-      </x:c>
-      <x:c r="V8" s="1798"/>
-      <x:c r="W8" s="1109"/>
-      <x:c r="X8" s="1108"/>
+        <x:f t="shared" ref="J8:J12" si="2">S8</x:f>
+      </x:c>
+      <x:c r="K8" s="1777" t="str">
+        <x:f t="shared" ref="K8:K12" si="3">IF(IF(ISNUMBER(E8),AND(E8&gt;=0,E8&lt;=3,MOD(E8,1)=0),FALSE),IF(E8=0,0,IF(IF(ISNUMBER(F8),AND(F8&gt;=1,F8&lt;=4,MOD(F8,1)=0),FALSE),E8*10+F8,"")),"")</x:f>
+      </x:c>
+      <x:c r="L8" s="1777" t="b">
+        <x:f t="shared" ref="L8:L12" si="4">IF(ISNUMBER(K8),K8=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="1777" t="b">
+        <x:f t="shared" ref="M8:M12" si="5">IF(ISNUMBER(K8),OR(K8=21,K8=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="1777" t="b">
+        <x:f t="shared" ref="N8:N12" si="6">IF(ISNUMBER(K8),OR(K8=22,K8=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="1777" t="b">
+        <x:f t="shared" ref="O8:O12" si="7">IF(ISNUMBER(K8),OR(K8=11,K8=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P8" s="1777" t="b">
+        <x:f t="shared" ref="P8:P12" si="8">IF(ISNUMBER(K8),OR(K8=23,K8=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="1777" t="b">
+        <x:f t="shared" ref="Q8:Q12" si="9">IF(ISNUMBER(K8),OR(K8=13,K8=14,K8=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R8" s="1777" t="b">
+        <x:f t="shared" ref="R8:R12" si="10">IF(ISNUMBER(K8),K8=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="1777" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T8),INDEX($L$5:$R$5,1,7-T8),"")</x:f>
+      </x:c>
+      <x:c r="T8" s="1777" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K8),IF(L8,6,IF(M8,5,IF(N8,4,IF(O8,3,IF(P8,2,IF(Q8,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U8" s="1790" t="str">
+        <x:f t="shared" ref="U8:U12" si="11">IF(AND(ISNUMBER(T8),ISNUMBER(H8)),IF(AND(H8&gt;=1,H8&lt;=4,MOD(H8,1)=0),T8*10+H8,""),"")</x:f>
+      </x:c>
+      <x:c r="V8" s="1799"/>
+      <x:c r="W8" s="1118"/>
+      <x:c r="X8" s="1117"/>
     </x:row>
     <x:row r="9" s="952" customFormat="1" ht="76" customHeight="1">
       <x:c r="A9" s="951"/>
@@ -42994,53 +42345,53 @@
       <x:c r="F9" s="1802"/>
       <x:c r="G9" s="1798"/>
       <x:c r="H9" s="1802"/>
-      <x:c r="I9" s="1798"/>
+      <x:c r="I9" s="1799"/>
       <x:c r="J9" s="1806" t="str">
-        <x:f t="shared" si="0">S9</x:f>
+        <x:f t="shared" si="2">S9</x:f>
       </x:c>
       <x:c r="K9" s="1783" t="str">
-        <x:f>IF(IF(ISNUMBER(E9),AND(E9&gt;=0,E9&lt;=3,MOD(E9,1)=0),FALSE),IF(E9=0,0,IF(IF(ISNUMBER(F9),AND(F9&gt;=1,F9&lt;=4,MOD(F9,1)=0),FALSE),E9*10+F9,"")),"")</x:f>
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E9),AND(E9&gt;=0,E9&lt;=3,MOD(E9,1)=0),FALSE),IF(E9=0,0,IF(IF(ISNUMBER(F9),AND(F9&gt;=1,F9&lt;=4,MOD(F9,1)=0),FALSE),E9*10+F9,"")),"")</x:f>
       </x:c>
       <x:c r="L9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),K9=31,FALSE)</x:f>
+        <x:f t="shared" si="4">IF(ISNUMBER(K9),K9=31,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=21,K9=32),FALSE)</x:f>
+        <x:f t="shared" si="5">IF(ISNUMBER(K9),OR(K9=21,K9=32),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=22,K9=33),FALSE)</x:f>
+        <x:f t="shared" si="6">IF(ISNUMBER(K9),OR(K9=22,K9=33),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=11,K9=12),FALSE)</x:f>
+        <x:f t="shared" si="7">IF(ISNUMBER(K9),OR(K9=11,K9=12),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=23,K9=34),FALSE)</x:f>
+        <x:f t="shared" si="8">IF(ISNUMBER(K9),OR(K9=23,K9=34),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),OR(K9=13,K9=14,K9=24),FALSE)</x:f>
+        <x:f t="shared" si="9">IF(ISNUMBER(K9),OR(K9=13,K9=14,K9=24),FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R9" s="1783" t="b">
-        <x:f>IF(ISNUMBER(K9),K9=0,FALSE)</x:f>
+        <x:f t="shared" si="10">IF(ISNUMBER(K9),K9=0,FALSE)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S9" s="1783" t="str">
-        <x:f>IF(ISNUMBER(T9),INDEX($L$5:$R$5,1,7-T9),"")</x:f>
+        <x:f t="shared" si="0">IF(ISNUMBER(T9),INDEX($L$5:$R$5,1,7-T9),"")</x:f>
       </x:c>
       <x:c r="T9" s="1783" t="str">
-        <x:f>IF(ISNUMBER(K9),IF(L9,6,IF(M9,5,IF(N9,4,IF(O9,3,IF(P9,2,IF(Q9,1,0)))))),"")</x:f>
+        <x:f t="shared" si="1">IF(ISNUMBER(K9),IF(L9,6,IF(M9,5,IF(N9,4,IF(O9,3,IF(P9,2,IF(Q9,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U9" s="1783" t="str">
-        <x:f>IF(AND(ISNUMBER(T9),ISNUMBER(H9)),IF(AND(H9&gt;=1,H9&lt;=4,MOD(H9,1)=0),T9*10+H9,""),"")</x:f>
-      </x:c>
-      <x:c r="V9" s="1798"/>
-      <x:c r="W9" s="1122"/>
-      <x:c r="X9" s="1114"/>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T9),ISNUMBER(H9)),IF(AND(H9&gt;=1,H9&lt;=4,MOD(H9,1)=0),T9*10+H9,""),"")</x:f>
+      </x:c>
+      <x:c r="V9" s="1799"/>
+      <x:c r="W9" s="1104"/>
+      <x:c r="X9" s="1116"/>
     </x:row>
     <x:row r="10" s="952" customFormat="1" ht="70" customHeight="1">
       <x:c r="A10" s="951"/>
@@ -43059,64 +42410,64 @@
       <x:c r="F10" s="1802"/>
       <x:c r="G10" s="1798"/>
       <x:c r="H10" s="1802"/>
-      <x:c r="I10" s="1798"/>
+      <x:c r="I10" s="1799"/>
       <x:c r="J10" s="1806" t="str">
-        <x:f>S10</x:f>
-      </x:c>
-      <x:c r="K10" s="1777" t="str">
-        <x:f>IF(IF(ISNUMBER(E10),AND(E10&gt;=0,E10&lt;=3,MOD(E10,1)=0),FALSE),IF(E10=0,0,IF(IF(ISNUMBER(F10),AND(F10&gt;=1,F10&lt;=4,MOD(F10,1)=0),FALSE),E10*10+F10,"")),"")</x:f>
-      </x:c>
-      <x:c r="L10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),K10=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=21,K10=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=22,K10=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=11,K10=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=23,K10=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),OR(K10=13,K10=14,K10=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R10" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K10),K10=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S10" s="1777" t="str">
-        <x:f>IF(ISNUMBER(T10),INDEX($L$5:$R$5,1,7-T10),"")</x:f>
-      </x:c>
-      <x:c r="T10" s="1777" t="str">
-        <x:f>IF(ISNUMBER(K10),IF(L10,6,IF(M10,5,IF(N10,4,IF(O10,3,IF(P10,2,IF(Q10,1,0)))))),"")</x:f>
+        <x:f t="shared" si="2">S10</x:f>
+      </x:c>
+      <x:c r="K10" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E10),AND(E10&gt;=0,E10&lt;=3,MOD(E10,1)=0),FALSE),IF(E10=0,0,IF(IF(ISNUMBER(F10),AND(F10&gt;=1,F10&lt;=4,MOD(F10,1)=0),FALSE),E10*10+F10,"")),"")</x:f>
+      </x:c>
+      <x:c r="L10" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K10),K10=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K10),OR(K10=21,K10=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K10),OR(K10=22,K10=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K10),OR(K10=11,K10=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P10" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K10),OR(K10=23,K10=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K10),OR(K10=13,K10=14,K10=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R10" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K10),K10=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T10),INDEX($L$5:$R$5,1,7-T10),"")</x:f>
+      </x:c>
+      <x:c r="T10" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K10),IF(L10,6,IF(M10,5,IF(N10,4,IF(O10,3,IF(P10,2,IF(Q10,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U10" s="1790" t="str">
-        <x:f>IF(AND(ISNUMBER(T10),ISNUMBER(H10)),IF(AND(H10&gt;=1,H10&lt;=4,MOD(H10,1)=0),T10*10+H10,""),"")</x:f>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T10),ISNUMBER(H10)),IF(AND(H10&gt;=1,H10&lt;=4,MOD(H10,1)=0),T10*10+H10,""),"")</x:f>
       </x:c>
       <x:c r="V10" s="1798"/>
-      <x:c r="W10" s="1109"/>
-      <x:c r="X10" s="1108"/>
+      <x:c r="W10" s="1105"/>
+      <x:c r="X10" s="903"/>
     </x:row>
-    <x:row r="11" s="952" customFormat="1" ht="70" customHeight="1">
+    <x:row r="11" s="952" customFormat="1" ht="100" customHeight="1">
       <x:c r="A11" s="951"/>
-      <x:c r="B11" s="1804" t="inlineStr">
+      <x:c r="B11" s="1805" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">C.5</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="1796" t="inlineStr">
+      <x:c r="C11" s="1797" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Former les élus et les agents au numérique responsable, et l'inscrire dans la stratégie numérique responsable prévue par la loi REEN.</x:t>
+          <x:t xml:space="preserve">Adopter et faire vivre la stratégie numérique responsable prévue par la loi REEN : obligatoire pour les communes et intercommunalités de plus de 50 000 habitants, recommandée pour les autres. Fixer des objectifs de réduction de l'empreinte du numérique, suivre leur mise en œuvre et former les élus et les agents.</x:t>
         </x:is>
       </x:c>
       <x:c r="D11" s="1798"/>
@@ -43124,98 +42475,289 @@
       <x:c r="F11" s="1802"/>
       <x:c r="G11" s="1798"/>
       <x:c r="H11" s="1802"/>
-      <x:c r="I11" s="1798"/>
-      <x:c r="J11" s="1806" t="n">
-        <x:f>S11</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K11" s="1777" t="str">
-        <x:f>IF(IF(ISNUMBER(E11),AND(E11&gt;=0,E11&lt;=3,MOD(E11,1)=0),FALSE),IF(E11=0,0,IF(IF(ISNUMBER(F11),AND(F11&gt;=1,F11&lt;=4,MOD(F11,1)=0),FALSE),E11*10+F11,"")),"")</x:f>
-      </x:c>
-      <x:c r="L11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),K11=31,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=21,K11=32),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=22,K11=33),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=11,K11=12),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=23,K11=34),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),OR(K11=13,K11=14,K11=24),FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R11" s="1777" t="b">
-        <x:f>IF(ISNUMBER(K11),K11=0,FALSE)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S11" s="1777" t="str">
-        <x:f>IF(ISNUMBER(T11),INDEX($L$5:$R$5,1,7-T11),"")</x:f>
-      </x:c>
-      <x:c r="T11" s="1777" t="str">
-        <x:f>IF(ISNUMBER(K11),IF(L11,6,IF(M11,5,IF(N11,4,IF(O11,3,IF(P11,2,IF(Q11,1,0)))))),"")</x:f>
+      <x:c r="I11" s="1799"/>
+      <x:c r="J11" s="1806" t="str">
+        <x:f t="shared" si="2">S11</x:f>
+      </x:c>
+      <x:c r="K11" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E11),AND(E11&gt;=0,E11&lt;=3,MOD(E11,1)=0),FALSE),IF(E11=0,0,IF(IF(ISNUMBER(F11),AND(F11&gt;=1,F11&lt;=4,MOD(F11,1)=0),FALSE),E11*10+F11,"")),"")</x:f>
+      </x:c>
+      <x:c r="L11" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K11),K11=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K11),OR(K11=21,K11=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K11),OR(K11=22,K11=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K11),OR(K11=11,K11=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P11" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K11),OR(K11=23,K11=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q11" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K11),OR(K11=13,K11=14,K11=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R11" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K11),K11=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T11),INDEX($L$5:$R$5,1,7-T11),"")</x:f>
+      </x:c>
+      <x:c r="T11" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K11),IF(L11,6,IF(M11,5,IF(N11,4,IF(O11,3,IF(P11,2,IF(Q11,1,0)))))),"")</x:f>
       </x:c>
       <x:c r="U11" s="1790" t="str">
-        <x:f>IF(AND(ISNUMBER(T11),ISNUMBER(H11)),IF(AND(H11&gt;=1,H11&lt;=4,MOD(H11,1)=0),T11*10+H11,""),"")</x:f>
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T11),ISNUMBER(H11)),IF(AND(H11&gt;=1,H11&lt;=4,MOD(H11,1)=0),T11*10+H11,""),"")</x:f>
       </x:c>
       <x:c r="V11" s="1798"/>
-      <x:c r="W11" s="1109"/>
-      <x:c r="X11" s="1108"/>
+      <x:c r="W11" s="1119"/>
+      <x:c r="X11" s="1114"/>
     </x:row>
-    <x:row r="12">
-      <x:c r="V12" s="893"/>
+    <x:row r="12" s="953" customFormat="1" ht="100" customHeight="1">
+      <x:c r="A12" s="951"/>
+      <x:c r="B12" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rendre accessibles les contenus que la collectivité produit chaque jour : documents, publications sur les réseaux sociaux, vidéos sous-titrées, textes en facile à lire et à comprendre (FALC). Former les agents qui les produisent et offrir un accueil accessible, y compris aux personnes sourdes et malentendantes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="1798"/>
+      <x:c r="E12" s="1802"/>
+      <x:c r="F12" s="1802"/>
+      <x:c r="G12" s="1798"/>
+      <x:c r="H12" s="1802"/>
+      <x:c r="I12" s="1799"/>
+      <x:c r="J12" s="1806" t="str">
+        <x:f t="shared" si="2">S12</x:f>
+      </x:c>
+      <x:c r="K12" s="1786" t="str">
+        <x:f t="shared" si="3">IF(IF(ISNUMBER(E12),AND(E12&gt;=0,E12&lt;=3,MOD(E12,1)=0),FALSE),IF(E12=0,0,IF(IF(ISNUMBER(F12),AND(F12&gt;=1,F12&lt;=4,MOD(F12,1)=0),FALSE),E12*10+F12,"")),"")</x:f>
+      </x:c>
+      <x:c r="L12" s="1786" t="b">
+        <x:f t="shared" si="4">IF(ISNUMBER(K12),K12=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="1786" t="b">
+        <x:f t="shared" si="5">IF(ISNUMBER(K12),OR(K12=21,K12=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="1786" t="b">
+        <x:f t="shared" si="6">IF(ISNUMBER(K12),OR(K12=22,K12=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="1786" t="b">
+        <x:f t="shared" si="7">IF(ISNUMBER(K12),OR(K12=11,K12=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P12" s="1786" t="b">
+        <x:f t="shared" si="8">IF(ISNUMBER(K12),OR(K12=23,K12=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q12" s="1786" t="b">
+        <x:f t="shared" si="9">IF(ISNUMBER(K12),OR(K12=13,K12=14,K12=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R12" s="1786" t="b">
+        <x:f t="shared" si="10">IF(ISNUMBER(K12),K12=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="1786" t="str">
+        <x:f t="shared" si="0">IF(ISNUMBER(T12),INDEX($L$5:$R$5,1,7-T12),"")</x:f>
+      </x:c>
+      <x:c r="T12" s="1786" t="str">
+        <x:f t="shared" si="1">IF(ISNUMBER(K12),IF(L12,6,IF(M12,5,IF(N12,4,IF(O12,3,IF(P12,2,IF(Q12,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U12" s="1790" t="str">
+        <x:f t="shared" si="11">IF(AND(ISNUMBER(T12),ISNUMBER(H12)),IF(AND(H12&gt;=1,H12&lt;=4,MOD(H12,1)=0),T12*10+H12,""),"")</x:f>
+      </x:c>
+      <x:c r="V12" s="1798"/>
+      <x:c r="W12" s="1120"/>
+      <x:c r="X12" s="1114"/>
+    </x:row>
+    <x:row r="13" ht="88.5" customHeight="1">
+      <x:c r="B13" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Recenser les usages de l'intelligence artificielle dans la collectivité, y compris l'IA générative utilisée par les agents. Les encadrer par une charte, vérifier les obligations du règlement européen sur l'IA, et informer les habitants des usages qui les concernent.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="1798"/>
+      <x:c r="E13" s="1802"/>
+      <x:c r="F13" s="1802"/>
+      <x:c r="G13" s="1798"/>
+      <x:c r="H13" s="1802"/>
+      <x:c r="I13" s="1799"/>
+      <x:c r="J13" s="1806" t="str">
+        <x:f t="shared" ref="J13" si="12">S13</x:f>
+      </x:c>
+      <x:c r="K13" s="1786" t="str">
+        <x:f t="shared" ref="K13" si="13">IF(IF(ISNUMBER(E13),AND(E13&gt;=0,E13&lt;=3,MOD(E13,1)=0),FALSE),IF(E13=0,0,IF(IF(ISNUMBER(F13),AND(F13&gt;=1,F13&lt;=4,MOD(F13,1)=0),FALSE),E13*10+F13,"")),"")</x:f>
+      </x:c>
+      <x:c r="L13" s="1786" t="b">
+        <x:f t="shared" ref="L13" si="14">IF(ISNUMBER(K13),K13=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="1786" t="b">
+        <x:f t="shared" ref="M13" si="15">IF(ISNUMBER(K13),OR(K13=21,K13=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="1786" t="b">
+        <x:f t="shared" ref="N13" si="16">IF(ISNUMBER(K13),OR(K13=22,K13=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="1786" t="b">
+        <x:f t="shared" ref="O13" si="17">IF(ISNUMBER(K13),OR(K13=11,K13=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P13" s="1786" t="b">
+        <x:f t="shared" ref="P13" si="18">IF(ISNUMBER(K13),OR(K13=23,K13=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q13" s="1786" t="b">
+        <x:f t="shared" ref="Q13" si="19">IF(ISNUMBER(K13),OR(K13=13,K13=14,K13=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R13" s="1786" t="b">
+        <x:f t="shared" ref="R13" si="20">IF(ISNUMBER(K13),K13=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="1786" t="str">
+        <x:f t="shared" ref="S13" si="21">IF(ISNUMBER(T13),INDEX($L$5:$R$5,1,7-T13),"")</x:f>
+      </x:c>
+      <x:c r="T13" s="1786" t="str">
+        <x:f t="shared" ref="T13" si="22">IF(ISNUMBER(K13),IF(L13,6,IF(M13,5,IF(N13,4,IF(O13,3,IF(P13,2,IF(Q13,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U13" s="1790" t="str">
+        <x:f t="shared" ref="U13" si="23">IF(AND(ISNUMBER(T13),ISNUMBER(H13)),IF(AND(H13&gt;=1,H13&lt;=4,MOD(H13,1)=0),T13*10+H13,""),"")</x:f>
+      </x:c>
+      <x:c r="V13" s="1798"/>
+      <x:c r="W13" s="1121"/>
+      <x:c r="X13" s="1114"/>
+    </x:row>
+    <x:row r="14" ht="88.5" customHeight="1">
+      <x:c r="B14" s="1804" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="1797" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Ouvrir la décision publique avec des outils de participation citoyenne (civic tech) : consultations, budgets participatifs, signalements. Choisir des outils ouverts, accessibles et sobres, comme les logiciels libres, et les compléter par des temps d'échange en présentiel.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="1798"/>
+      <x:c r="E14" s="1802"/>
+      <x:c r="F14" s="1802"/>
+      <x:c r="G14" s="1798"/>
+      <x:c r="H14" s="1802"/>
+      <x:c r="I14" s="1799"/>
+      <x:c r="J14" s="1806" t="n">
+        <x:f>S14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" s="1786" t="str">
+        <x:f>IF(IF(ISNUMBER(E14),AND(E14&gt;=0,E14&lt;=3,MOD(E14,1)=0),FALSE),IF(E14=0,0,IF(IF(ISNUMBER(F14),AND(F14&gt;=1,F14&lt;=4,MOD(F14,1)=0),FALSE),E14*10+F14,"")),"")</x:f>
+      </x:c>
+      <x:c r="L14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),K14=31,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=21,K14=32),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=22,K14=33),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=11,K14=12),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=23,K14=34),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),OR(K14=13,K14=14,K14=24),FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R14" s="1786" t="b">
+        <x:f>IF(ISNUMBER(K14),K14=0,FALSE)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S14" s="1786" t="str">
+        <x:f>IF(ISNUMBER(T14),INDEX($L$5:$R$5,1,7-T14),"")</x:f>
+      </x:c>
+      <x:c r="T14" s="1786" t="str">
+        <x:f>IF(ISNUMBER(K14),IF(L14,6,IF(M14,5,IF(N14,4,IF(O14,3,IF(P14,2,IF(Q14,1,0)))))),"")</x:f>
+      </x:c>
+      <x:c r="U14" s="1790" t="str">
+        <x:f>IF(AND(ISNUMBER(T14),ISNUMBER(H14)),IF(AND(H14&gt;=1,H14&lt;=4,MOD(H14,1)=0),T14*10+H14,""),"")</x:f>
+      </x:c>
+      <x:c r="V14" s="1798"/>
+      <x:c r="W14" s="1121"/>
+      <x:c r="X14" s="1114"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="V4:X4"/>
+    <x:mergeCell ref="B6:W6"/>
     <x:mergeCell ref="B4:C5"/>
     <x:mergeCell ref="D4:E4"/>
     <x:mergeCell ref="F4:G4"/>
     <x:mergeCell ref="H4:I4"/>
+    <x:mergeCell ref="V4:X4"/>
     <x:mergeCell ref="B2:J3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="J7:J11">
-    <x:cfRule type="expression" dxfId="1633" priority="498">
+  <x:conditionalFormatting sqref="J7:J14">
+    <x:cfRule type="expression" dxfId="1626" priority="271">
       <x:formula>AND(ISNUMBER($T7),$T7=6)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1634" priority="499">
+    <x:cfRule type="expression" dxfId="1627" priority="272">
       <x:formula>AND(ISNUMBER($T7),$T7=5)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1635" priority="500">
+    <x:cfRule type="expression" dxfId="1628" priority="273">
       <x:formula>AND(ISNUMBER($T7),$T7=4)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1636" priority="501">
+    <x:cfRule type="expression" dxfId="1629" priority="274">
       <x:formula>AND(ISNUMBER($T7),$T7=3)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1637" priority="502">
+    <x:cfRule type="expression" dxfId="1630" priority="275">
       <x:formula>AND(ISNUMBER($T7),$T7=2)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1638" priority="503">
+    <x:cfRule type="expression" dxfId="1631" priority="276">
       <x:formula>AND(ISNUMBER($T7),$T7=1)</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1639" priority="504">
+    <x:cfRule type="expression" dxfId="1632" priority="277">
       <x:formula>AND(ISNUMBER($T7),$T7=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="E7:E11" promptTitle="Importance de la cible" prompt="0 : non applicable&#10;1 : peu importante&#10;2 : importante&#10;3 : très importante&#10;Si 0, la performance peut rester vide." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="E7:E14" promptTitle="Importance de la cible" prompt="0 : non applicable&#10;1 : peu importante&#10;2 : importante&#10;3 : très importante&#10;Si 0, la performance peut rester vide." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"0,1,2,3"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="F7:F11" promptTitle="Performance actuelle" prompt="1 : pas du tout atteinte&#10;2 : atteinte en partie&#10;3 : en voie d’être atteinte&#10;4 : atteinte&#10;Laisser vide si non évaluée ou non applicable." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="F7:F14" promptTitle="Performance actuelle" prompt="1 : pas du tout atteinte&#10;2 : atteinte en partie&#10;3 : en voie d’être atteinte&#10;4 : atteinte&#10;Laisser vide si non évaluée ou non applicable." errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"1,2,3,4"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="H7:H11" promptTitle="Compétences mobilisées" prompt="1 : équipe NR / RSE&#10;2 : NR / RSE et DSI&#10;3 : NR / RSE et équipe hors DSI&#10;4 : intervention extérieure" errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" showDropDown="0" sqref="H7:H14" promptTitle="Compétences mobilisées" prompt="1 : équipe NR / RSE&#10;2 : NR / RSE et DSI&#10;3 : NR / RSE et équipe hors DSI&#10;4 : intervention extérieure" errorTitle="Note invalide" error="Choisir une note dans la liste ou laisser la cellule vide.">
       <x:formula1>"1,2,3,4"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
fix(classeurs): aligner les bandeaux de logos hors du texte
Le générateur place le bandeau dans une zone libre propre à chaque feuille
(ZONES_BANDEAU) au lieu d'ancres fixes : à droite du titre et calé sur le
bord du tableau (ONR, Cibles métier), dans le cadre du titre (synthèse,
résultats détaillés), sur une ligne dédiée (Contexte), en haut du cadre
centré (Accueil) ou au-dessus du texte (Méthodologie). Le bandeau prend la
plus grande taille qui tient dans sa zone, avec une marge de 1,5 mm.
positions_colonnes ignore désormais les colonnes masquées.

Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
+++ b/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
@@ -27567,12 +27567,12 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>76199</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>24037</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>104774</xdr:rowOff>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3600000" cy="540000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30039,11 +30039,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123824</xdr:colOff>
+      <xdr:colOff>120014</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>47624</xdr:rowOff>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3873146" cy="580972"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30273,12 +30273,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30365,12 +30365,12 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>650874</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>266699</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>483967</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3005333" cy="450800"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30430,9 +30430,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>7156450</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:colOff>4235425</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>55562</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
@@ -30461,12 +30461,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30493,12 +30493,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30525,12 +30525,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30557,12 +30557,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30589,12 +30589,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30621,10 +30621,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>212725</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1273150</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2076425</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
@@ -42472,7 +42472,7 @@
     <col min="16132" max="16384" width="10.6640625" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="6.75" customHeight="1"/>
+    <row r="1" spans="2:3" ht="59" customHeight="1"/>
     <row r="2" spans="2:3" ht="70.5" customHeight="1">
       <c r="B2" s="326" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
fix(classeurs): aligner les bandeaux de logos hors du texte (#17)
Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
+++ b/secteurs/collectivites/GPC-ONR_collectivites_Template.xlsx
@@ -27567,12 +27567,12 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>76199</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>24037</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>104774</xdr:rowOff>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3600000" cy="540000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30039,11 +30039,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123824</xdr:colOff>
+      <xdr:colOff>120014</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>47624</xdr:rowOff>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3873146" cy="580972"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30273,12 +30273,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30365,12 +30365,12 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>650874</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>266699</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>483967</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3005333" cy="450800"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30430,9 +30430,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>7156450</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:colOff>4235425</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>55562</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
@@ -30461,12 +30461,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30493,12 +30493,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30525,12 +30525,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30557,12 +30557,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30589,12 +30589,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>54002</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>117399</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4254500" cy="638175"/>
+    <xdr:ext cx="3006673" cy="451001"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Logos INR, LaNum Pays Basque et NÉONUM"/>
@@ -30621,10 +30621,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>212725</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1273150</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2076425</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4254500" cy="638175"/>
     <xdr:pic>
@@ -42472,7 +42472,7 @@
     <col min="16132" max="16384" width="10.6640625" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="6.75" customHeight="1"/>
+    <row r="1" spans="2:3" ht="59" customHeight="1"/>
     <row r="2" spans="2:3" ht="70.5" customHeight="1">
       <c r="B2" s="326" t="s">
         <v>1</v>

</xml_diff>